<commit_message>
1차 실험 완료 (SR, GCR, Exec)
</commit_message>
<xml_diff>
--- a/FP216_result.xlsx
+++ b/FP216_result.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -445,6 +445,8 @@
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,10 +472,20 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Physical Guard Exec (%)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Baseline Exec (%)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Physical Guard Status</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Baseline Status</t>
         </is>
@@ -482,43 +494,183 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Put Keychain and CreditCard into the box</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>100</v>
+      </c>
+      <c r="C2" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E2" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>77.78</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>FAILED (Execution Errors)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>FAILED (Execution Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Put the remotecontrol and creditcard and keychain in the box</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B3" t="n">
         <v>66.67</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C3" t="n">
         <v>33.33</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D3" t="n">
         <v>33.34</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="n">
+        <v>68.75</v>
+      </c>
+      <c r="F3" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>FAILED (Execution Errors)</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>FAILED (Execution Errors)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Turn off the Desklamp and Turn on the Laptop</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-100</v>
+      </c>
+      <c r="E4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F4" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>FAILED (Execution Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Turn off the floorlamp and desklamp</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>100</v>
+      </c>
+      <c r="C5" t="n">
+        <v>100</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F5" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>FAILED (Execution Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Turn on the Television</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>100</v>
+      </c>
+      <c r="C6" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>FAILED (Execution Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>평균</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>66.67</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>33.33</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>33.34</v>
+      <c r="B8" s="2" t="n">
+        <v>73.33</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>76.67</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>-3.33</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>91.25</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>86.39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>